<commit_message>
implements feedback to modify existing solution
</commit_message>
<xml_diff>
--- a/api/src/excelreports/reportTemplates/Supplies.xlsx
+++ b/api/src/excelreports/reportTemplates/Supplies.xlsx
@@ -339,7 +339,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -348,15 +348,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -788,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.5" customWidth="1"/>
@@ -803,11 +794,11 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="5" t="s">
         <v>35</v>
       </c>
     </row>
@@ -816,74 +807,169 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="11" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
+      <c r="B6"/>
+      <c r="C6"/>
+      <c r="D6"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
+      <c r="B9"/>
+      <c r="C9"/>
+      <c r="D9"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
+      <c r="B10"/>
+      <c r="C10"/>
+      <c r="D10"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11"/>
+      <c r="C11"/>
+      <c r="D11"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13"/>
+      <c r="C13"/>
+      <c r="D13"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B15"/>
+      <c r="C15"/>
+      <c r="D15"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18"/>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19"/>
+      <c r="C19"/>
+      <c r="D19"/>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20"/>
+      <c r="C20"/>
+      <c r="D20"/>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25"/>
+      <c r="C25"/>
+      <c r="D25"/>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26"/>
+      <c r="C26"/>
+      <c r="D26"/>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27"/>
+      <c r="C27"/>
+      <c r="D27"/>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B28"/>
+      <c r="C28"/>
+      <c r="D28"/>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29"/>
+      <c r="C29"/>
+      <c r="D29"/>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30"/>
+      <c r="C30"/>
+      <c r="D30"/>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31"/>
+      <c r="C31"/>
+      <c r="D31"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>